<commit_message>
first round report. Partial replication due to computational limitations. Minor issues with citations, and README
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,22 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/damandhaliwal/Documents/Research Work/JPE/Replications/Hansen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F310CDD6-AD12-7641-8607-C1BF8AB271B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40100" yWindow="600" windowWidth="20060" windowHeight="32500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="105">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -46,13 +57,307 @@
   </si>
   <si>
     <t>In-text numbers</t>
+  </si>
+  <si>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>Figure 3a</t>
+  </si>
+  <si>
+    <t>Figure 3b</t>
+  </si>
+  <si>
+    <t>Figure 4a</t>
+  </si>
+  <si>
+    <t>Figure 4b</t>
+  </si>
+  <si>
+    <t>Figure 5a</t>
+  </si>
+  <si>
+    <t>Figure 5b</t>
+  </si>
+  <si>
+    <t>Figure 6</t>
+  </si>
+  <si>
+    <t>Figure 7</t>
+  </si>
+  <si>
+    <t>Figure 8</t>
+  </si>
+  <si>
+    <t>Figure 9a</t>
+  </si>
+  <si>
+    <t>Figure 9b</t>
+  </si>
+  <si>
+    <t>Figure 9c</t>
+  </si>
+  <si>
+    <t>Figure 9d</t>
+  </si>
+  <si>
+    <t>Figure 10</t>
+  </si>
+  <si>
+    <t>Figure 11</t>
+  </si>
+  <si>
+    <t>Figure 12a</t>
+  </si>
+  <si>
+    <t>Figure 12b</t>
+  </si>
+  <si>
+    <t>Figure 13a</t>
+  </si>
+  <si>
+    <t>Figure 13b</t>
+  </si>
+  <si>
+    <t>Figure 14a</t>
+  </si>
+  <si>
+    <t>Figure 14b</t>
+  </si>
+  <si>
+    <t>Figure 15a</t>
+  </si>
+  <si>
+    <t>Figure 15b</t>
+  </si>
+  <si>
+    <t>Figure 16a</t>
+  </si>
+  <si>
+    <t>Figure 16b</t>
+  </si>
+  <si>
+    <t>Figure 16c</t>
+  </si>
+  <si>
+    <t>Figure 16d</t>
+  </si>
+  <si>
+    <t>Figure 17a</t>
+  </si>
+  <si>
+    <t>Figure 17b</t>
+  </si>
+  <si>
+    <t>Figure 17c</t>
+  </si>
+  <si>
+    <t>Figure 17d</t>
+  </si>
+  <si>
+    <t>Figure 18a</t>
+  </si>
+  <si>
+    <t>Figure 18b</t>
+  </si>
+  <si>
+    <t>Figure 18c</t>
+  </si>
+  <si>
+    <t>Figure 18d</t>
+  </si>
+  <si>
+    <t>Figure 19</t>
+  </si>
+  <si>
+    <t>Figure 20</t>
+  </si>
+  <si>
+    <t>Figure 21a</t>
+  </si>
+  <si>
+    <t>Figure 21b</t>
+  </si>
+  <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t>Table 3</t>
+  </si>
+  <si>
+    <t>Table 4</t>
+  </si>
+  <si>
+    <t>Table 5</t>
+  </si>
+  <si>
+    <t>Table 6</t>
+  </si>
+  <si>
+    <t>Table 7</t>
+  </si>
+  <si>
+    <t>Table 8</t>
+  </si>
+  <si>
+    <t>Table 9</t>
+  </si>
+  <si>
+    <t>Table 10</t>
+  </si>
+  <si>
+    <t>Table 11</t>
+  </si>
+  <si>
+    <t>Table 12</t>
+  </si>
+  <si>
+    <t>Table 13</t>
+  </si>
+  <si>
+    <t>Table 14</t>
+  </si>
+  <si>
+    <t>Table 15</t>
+  </si>
+  <si>
+    <t>Table 16</t>
+  </si>
+  <si>
+    <t>Table 17</t>
+  </si>
+  <si>
+    <t>Table 18</t>
+  </si>
+  <si>
+    <t>Table 19</t>
+  </si>
+  <si>
+    <t>Table 20</t>
+  </si>
+  <si>
+    <t>Table 21</t>
+  </si>
+  <si>
+    <t>Table 22</t>
+  </si>
+  <si>
+    <t>Table 23</t>
+  </si>
+  <si>
+    <t>Table 24</t>
+  </si>
+  <si>
+    <t>Table 25</t>
+  </si>
+  <si>
+    <t>pysrc/scripts/figure1.py</t>
+  </si>
+  <si>
+    <t>rsrc/analysis/carbon_capture_curves/02_analysis.R</t>
+  </si>
+  <si>
+    <t>rsrc/analysis/calibration_maps_1043_sites.R</t>
+  </si>
+  <si>
+    <t>pysrc/analysis/figures.py</t>
+  </si>
+  <si>
+    <t>rsrc/analysis/map_1043_det.R</t>
+  </si>
+  <si>
+    <t>pysrc/analysis/map.py</t>
+  </si>
+  <si>
+    <t>pysrc/scripts/mpc_trajectory.py</t>
+  </si>
+  <si>
+    <t>pysrc/scripts/price_estimation.py</t>
+  </si>
+  <si>
+    <t>rsrc/analysis/map_kl.R</t>
+  </si>
+  <si>
+    <t>rsrc/analysis/map_1043_hmc_xi1.R</t>
+  </si>
+  <si>
+    <t>rsrc/analysis/map_1043_hmc_xi05.R</t>
+  </si>
+  <si>
+    <t>pysrc/scripts/bayesian_R2.py</t>
+  </si>
+  <si>
+    <t>pysrc/replication/derive_carbon_prices.py</t>
+  </si>
+  <si>
+    <t>pysrc/analysis/tables.py</t>
+  </si>
+  <si>
+    <t>pysrc/mpc/mpc_compute_day0.py</t>
+  </si>
+  <si>
+    <t>pysrc/replication/derive_mpc_transition_probabilities.py</t>
+  </si>
+  <si>
+    <t>pysrc/mpc/mpc_compute_day0.py; pysrc/mpc/mpc_compute.py</t>
+  </si>
+  <si>
+    <t>462; 178</t>
+  </si>
+  <si>
+    <t>pysrc/sampling/baseline.py</t>
+  </si>
+  <si>
+    <t>Pg 17, Footnote 28 R^2</t>
+  </si>
+  <si>
+    <t>Pg 18, correlation is -0.27</t>
+  </si>
+  <si>
+    <t>Pg 24, footnote 35, when we move from 2 to 3 percent</t>
+  </si>
+  <si>
+    <t>Pg 39, Footnote 43</t>
+  </si>
+  <si>
+    <t>Pg 38, b = 25, bf = .15b, tau_f =15</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>rsrc/cleaning/_masterfile.R</t>
+  </si>
+  <si>
+    <t>rsrc/processing/_masterfile.R</t>
+  </si>
+  <si>
+    <t>rsrc/calibration/_masterfile.R</t>
+  </si>
+  <si>
+    <t>data/clean/: cleaned source-specific Rdata and raster files</t>
+  </si>
+  <si>
+    <t>data/processed/: cattle_price_index.Rdata; pixel_sample.Rdata; pixel_areas.Rdata; pixel_categories.Rdata; pixel_primary_forest_2017.Rdata; pixel_biomass_2017.Rdata; spatial, cross-section, and panel municipality samples; muni_biomass_2017.Rdata; muni_data.Rdata; state_emissions.Rdata; processed land-use and biome rasters</t>
+  </si>
+  <si>
+    <t>data/calibration/: calibration_1043_sites.Rdata/.csv; grid_1043_sites.geojson; calibration_78_sites.Rdata/.csv; grid_78_sites.geojson; gamma/theta calibration objects and fitted GeoJSON inputs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -67,6 +372,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -89,7 +400,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -99,6 +410,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -434,11 +751,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -461,47 +778,1067 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
+      <c r="A2" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="A3" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9">
+        <v>166</v>
+      </c>
+      <c r="D9" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10">
+        <v>68</v>
+      </c>
+      <c r="D10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11">
+        <v>104</v>
+      </c>
+      <c r="D11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12">
+        <v>195</v>
+      </c>
+      <c r="D12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13">
+        <v>225</v>
+      </c>
+      <c r="D13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14">
+        <v>246</v>
+      </c>
+      <c r="D14" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15">
+        <v>116</v>
+      </c>
+      <c r="D15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16">
+        <v>161</v>
+      </c>
+      <c r="D16" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17">
+        <v>557</v>
+      </c>
+      <c r="D17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18">
+        <v>305</v>
+      </c>
+      <c r="D18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19">
+        <v>353</v>
+      </c>
+      <c r="D19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20">
+        <v>374</v>
+      </c>
+      <c r="D20" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21">
+        <v>313</v>
+      </c>
+      <c r="D21" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22">
+        <v>404</v>
+      </c>
+      <c r="D22" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23">
+        <v>344</v>
+      </c>
+      <c r="D23" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24">
+        <v>114</v>
+      </c>
+      <c r="D24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25">
+        <v>482</v>
+      </c>
+      <c r="D25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26">
+        <v>114</v>
+      </c>
+      <c r="D26" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27">
+        <v>114</v>
+      </c>
+      <c r="D27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28">
+        <v>483</v>
+      </c>
+      <c r="D28" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29">
+        <v>483</v>
+      </c>
+      <c r="D29" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30">
+        <v>117</v>
+      </c>
+      <c r="D30" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31">
+        <v>117</v>
+      </c>
+      <c r="D31" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32">
+        <v>130</v>
+      </c>
+      <c r="D32" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>80</v>
+      </c>
+      <c r="C33">
+        <v>130</v>
+      </c>
+      <c r="D33" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34">
+        <v>352</v>
+      </c>
+      <c r="D34" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>81</v>
+      </c>
+      <c r="C35">
+        <v>366</v>
+      </c>
+      <c r="D35" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
+        <v>81</v>
+      </c>
+      <c r="C36">
+        <v>359</v>
+      </c>
+      <c r="D36" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
+        <v>81</v>
+      </c>
+      <c r="C37">
+        <v>373</v>
+      </c>
+      <c r="D37" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38">
+        <v>374</v>
+      </c>
+      <c r="D38" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>37</v>
+      </c>
+      <c r="B39" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39">
+        <v>313</v>
+      </c>
+      <c r="D39" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" t="s">
+        <v>76</v>
+      </c>
+      <c r="C40">
+        <v>404</v>
+      </c>
+      <c r="D40" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" t="s">
+        <v>76</v>
+      </c>
+      <c r="C41">
+        <v>344</v>
+      </c>
+      <c r="D41" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42">
+        <v>374</v>
+      </c>
+      <c r="D42" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
+        <v>76</v>
+      </c>
+      <c r="C43">
+        <v>313</v>
+      </c>
+      <c r="D43" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
+        <v>76</v>
+      </c>
+      <c r="C44">
+        <v>404</v>
+      </c>
+      <c r="D44" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" t="s">
+        <v>76</v>
+      </c>
+      <c r="C45">
+        <v>344</v>
+      </c>
+      <c r="D45" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" t="s">
+        <v>82</v>
+      </c>
+      <c r="C46">
+        <v>317</v>
+      </c>
+      <c r="D46" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47" t="s">
+        <v>83</v>
+      </c>
+      <c r="C47">
+        <v>298</v>
+      </c>
+      <c r="D47" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>46</v>
+      </c>
+      <c r="B48" t="s">
+        <v>84</v>
+      </c>
+      <c r="C48">
+        <v>70</v>
+      </c>
+      <c r="D48" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>47</v>
+      </c>
+      <c r="B49" t="s">
+        <v>84</v>
+      </c>
+      <c r="C49">
+        <v>108</v>
+      </c>
+      <c r="D49" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" t="s">
+        <v>85</v>
+      </c>
+      <c r="C50">
+        <v>275</v>
+      </c>
+      <c r="D50" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>49</v>
+      </c>
+      <c r="B51" t="s">
+        <v>86</v>
+      </c>
+      <c r="C51">
+        <v>136</v>
+      </c>
+      <c r="D51" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>50</v>
+      </c>
+      <c r="B52" t="s">
+        <v>86</v>
+      </c>
+      <c r="C52">
+        <v>253</v>
+      </c>
+      <c r="D52" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>51</v>
+      </c>
+      <c r="B53" t="s">
+        <v>86</v>
+      </c>
+      <c r="C53">
+        <v>454</v>
+      </c>
+      <c r="D53" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>52</v>
+      </c>
+      <c r="B54" t="s">
+        <v>85</v>
+      </c>
+      <c r="C54">
+        <v>275</v>
+      </c>
+      <c r="D54" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>53</v>
+      </c>
+      <c r="B55" t="s">
+        <v>87</v>
+      </c>
+      <c r="C55">
+        <v>462</v>
+      </c>
+      <c r="D55" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>54</v>
+      </c>
+      <c r="B56" t="s">
+        <v>88</v>
+      </c>
+      <c r="C56">
+        <v>305</v>
+      </c>
+      <c r="D56" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>55</v>
+      </c>
+      <c r="B57" t="s">
+        <v>87</v>
+      </c>
+      <c r="C57">
+        <v>462</v>
+      </c>
+      <c r="D57" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>56</v>
+      </c>
+      <c r="B58" t="s">
+        <v>88</v>
+      </c>
+      <c r="C58">
+        <v>305</v>
+      </c>
+      <c r="D58" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>57</v>
+      </c>
+      <c r="B59" t="s">
+        <v>80</v>
+      </c>
+      <c r="C59">
+        <v>263</v>
+      </c>
+      <c r="D59" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>58</v>
+      </c>
+      <c r="B60" t="s">
+        <v>80</v>
+      </c>
+      <c r="C60">
+        <v>267</v>
+      </c>
+      <c r="D60" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61" t="s">
+        <v>87</v>
+      </c>
+      <c r="C61">
+        <v>462</v>
+      </c>
+      <c r="D61" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>60</v>
+      </c>
+      <c r="B62" t="s">
+        <v>86</v>
+      </c>
+      <c r="C62">
+        <v>136</v>
+      </c>
+      <c r="D62" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>61</v>
+      </c>
+      <c r="B63" t="s">
+        <v>86</v>
+      </c>
+      <c r="C63">
+        <v>258</v>
+      </c>
+      <c r="D63" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>62</v>
+      </c>
+      <c r="B64" t="s">
+        <v>86</v>
+      </c>
+      <c r="C64">
+        <v>258</v>
+      </c>
+      <c r="D64" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>63</v>
+      </c>
+      <c r="B65" t="s">
+        <v>86</v>
+      </c>
+      <c r="C65">
+        <v>454</v>
+      </c>
+      <c r="D65" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>64</v>
+      </c>
+      <c r="B66" t="s">
+        <v>86</v>
+      </c>
+      <c r="C66">
+        <v>454</v>
+      </c>
+      <c r="D66" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>65</v>
+      </c>
+      <c r="B67" t="s">
+        <v>89</v>
+      </c>
+      <c r="C67" t="s">
+        <v>90</v>
+      </c>
+      <c r="D67" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>66</v>
+      </c>
+      <c r="B68" t="s">
+        <v>87</v>
+      </c>
+      <c r="C68">
+        <v>462</v>
+      </c>
+      <c r="D68" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>67</v>
+      </c>
+      <c r="B69" t="s">
+        <v>88</v>
+      </c>
+      <c r="C69">
+        <v>305</v>
+      </c>
+      <c r="D69" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>68</v>
+      </c>
+      <c r="B70" t="s">
+        <v>87</v>
+      </c>
+      <c r="C70">
+        <v>462</v>
+      </c>
+      <c r="D70" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>69</v>
+      </c>
+      <c r="B71" t="s">
+        <v>88</v>
+      </c>
+      <c r="C71">
+        <v>305</v>
+      </c>
+      <c r="D71" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>70</v>
+      </c>
+      <c r="B72" t="s">
+        <v>91</v>
+      </c>
+      <c r="C72">
+        <v>127</v>
+      </c>
+      <c r="D72" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>71</v>
+      </c>
+      <c r="B73" t="s">
+        <v>91</v>
+      </c>
+      <c r="C73">
+        <v>116</v>
+      </c>
+      <c r="D73" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>72</v>
+      </c>
+      <c r="B74" t="s">
+        <v>91</v>
+      </c>
+      <c r="C74">
+        <v>149</v>
+      </c>
+      <c r="D74" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B76" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C76" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D76" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>2</v>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>92</v>
+      </c>
+      <c r="B77" t="s">
+        <v>98</v>
+      </c>
+      <c r="C77" t="s">
+        <v>98</v>
+      </c>
+      <c r="D77" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>93</v>
+      </c>
+      <c r="B78" t="s">
+        <v>98</v>
+      </c>
+      <c r="C78" t="s">
+        <v>98</v>
+      </c>
+      <c r="D78" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>94</v>
+      </c>
+      <c r="B79" t="s">
+        <v>98</v>
+      </c>
+      <c r="C79" t="s">
+        <v>98</v>
+      </c>
+      <c r="D79" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>96</v>
+      </c>
+      <c r="B80" t="s">
+        <v>98</v>
+      </c>
+      <c r="C80" t="s">
+        <v>98</v>
+      </c>
+      <c r="D80" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>95</v>
+      </c>
+      <c r="B81" t="s">
+        <v>98</v>
+      </c>
+      <c r="C81" t="s">
+        <v>98</v>
+      </c>
+      <c r="D81" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>